<commit_message>
feat - fix bulk drum delete message, support CSV import, and add container_no column
</commit_message>
<xml_diff>
--- a/public/drum-import-template.xlsx
+++ b/public/drum-import-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anthonyshoshigomes/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kishorbiswas/NSS/drum-delivery-web/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EE898B5-1C74-EE43-A342-A34C434F216A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5813A392-9AD2-C34E-B234-2A8357494BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{12FDB0EE-E9FD-0142-B20E-B744DFC80197}"/>
+    <workbookView xWindow="-38400" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{12FDB0EE-E9FD-0142-B20E-B744DFC80197}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>drum_number</t>
   </si>
@@ -63,13 +62,22 @@
   </si>
   <si>
     <t>DR002</t>
+  </si>
+  <si>
+    <t>container_no</t>
+  </si>
+  <si>
+    <t>ABC123</t>
+  </si>
+  <si>
+    <t>ABC124</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -81,6 +89,12 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -443,67 +457,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC790935-8B1E-4C43-881B-1338AE8DEC5F}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2">
         <v>12.5</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>100</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>110</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
       <c r="C3">
+        <v>10</v>
+      </c>
+      <c r="D3">
         <v>90</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>95</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>